<commit_message>
feat(phase-75): multi-enterprise governance and portfolio operating model (ADR 0044)
</commit_message>
<xml_diff>
--- a/DOCUMENTACION/AI_OPERATING_PLATFORM_BACKLOG_KANBAN.xlsx
+++ b/DOCUMENTACION/AI_OPERATING_PLATFORM_BACKLOG_KANBAN.xlsx
@@ -539,7 +539,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H49"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -1346,7 +1346,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -1484,7 +1484,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -1811,7 +1811,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
@@ -2865,7 +2865,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -3275,7 +3275,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
@@ -3714,7 +3714,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O50"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -7380,7 +7380,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -7986,7 +7986,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
@@ -8624,7 +8624,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -9315,7 +9315,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
@@ -9536,7 +9536,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -10048,7 +10048,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -10418,7 +10418,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>

</xml_diff>